<commit_message>
27 November 2025 from home
</commit_message>
<xml_diff>
--- a/SUPPLIER RELATED/Phone Book BALAGAN.xlsx
+++ b/SUPPLIER RELATED/Phone Book BALAGAN.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7500"/>
+    <workbookView windowHeight="17000"/>
   </bookViews>
   <sheets>
     <sheet name="Contact lists" sheetId="1" r:id="rId1"/>
@@ -97,7 +97,7 @@
 Estimulo malbec
 Fashion vodka
 McGuigan
-CAmpari
+Campari
 Vitral syrah
 Dona dominga
 Rose pipoli
@@ -138,7 +138,6 @@
 Jagermeister
 Grey goose
 McGuigan
-Campari
 Jim beam black / white
 Herradura
 Mancino rosso
@@ -661,10 +660,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -833,12 +832,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
@@ -1183,16 +1182,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1696,13 +1695,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E69"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="5.08571428571429" style="2" customWidth="1"/>
-    <col min="2" max="2" width="29.4285714285714" customWidth="1"/>
-    <col min="3" max="3" width="33.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="17.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="46.1809523809524" customWidth="1"/>
+    <col min="1" max="1" width="5.0859375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="29.4296875" customWidth="1"/>
+    <col min="3" max="3" width="33.4296875" customWidth="1"/>
+    <col min="4" max="4" width="17.859375" customWidth="1"/>
+    <col min="5" max="5" width="46.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">

</xml_diff>

<commit_message>
6 DECEMBER 2025 CLOSING
</commit_message>
<xml_diff>
--- a/SUPPLIER RELATED/Phone Book BALAGAN.xlsx
+++ b/SUPPLIER RELATED/Phone Book BALAGAN.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17000"/>
+    <workbookView windowWidth="19635" windowHeight="7500"/>
   </bookViews>
   <sheets>
     <sheet name="Contact lists" sheetId="1" r:id="rId1"/>
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="172">
   <si>
     <t>BALAGAN RESTO &amp; LOUNGE BAR</t>
   </si>
@@ -653,6 +653,21 @@
   </si>
   <si>
     <t>+62 877-2913-3528</t>
+  </si>
+  <si>
+    <t>Abiseka 2nd</t>
+  </si>
+  <si>
+    <t>Fresh milk</t>
+  </si>
+  <si>
+    <t>081703200100</t>
+  </si>
+  <si>
+    <t>Dairy fresh milk 1st</t>
+  </si>
+  <si>
+    <t>089529399287</t>
   </si>
 </sst>
 </file>
@@ -660,10 +675,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -832,12 +847,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
@@ -1182,16 +1197,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1322,7 +1337,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1371,10 +1386,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1694,14 +1711,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E69"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="4"/>
+  <dimension ref="A1:E71"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="5.0859375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="29.4296875" customWidth="1"/>
-    <col min="3" max="3" width="33.4296875" customWidth="1"/>
-    <col min="4" max="4" width="17.859375" customWidth="1"/>
-    <col min="5" max="5" width="46.1796875" customWidth="1"/>
+    <col min="1" max="1" width="5.08571428571429" style="2" customWidth="1"/>
+    <col min="2" max="2" width="29.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="33.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="17.8571428571429" customWidth="1"/>
+    <col min="5" max="5" width="46.1809523809524" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1807,7 +1824,7 @@
       <c r="C10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="10"/>
@@ -1870,7 +1887,7 @@
       <c r="C16" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="10" t="s">
@@ -1902,7 +1919,7 @@
       <c r="C18" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="19" t="s">
         <v>31</v>
       </c>
       <c r="E18" s="10"/>
@@ -2117,7 +2134,7 @@
       <c r="C34" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="D34" s="19" t="s">
+      <c r="D34" s="20" t="s">
         <v>66</v>
       </c>
       <c r="E34" s="10" t="s">
@@ -2134,7 +2151,7 @@
       <c r="C35" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D35" s="19" t="s">
+      <c r="D35" s="20" t="s">
         <v>70</v>
       </c>
       <c r="E35" s="10" t="s">
@@ -2151,7 +2168,7 @@
       <c r="C36" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="19" t="s">
+      <c r="D36" s="20" t="s">
         <v>73</v>
       </c>
       <c r="E36" s="10" t="s">
@@ -2168,7 +2185,7 @@
       <c r="C37" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="D37" s="19" t="s">
+      <c r="D37" s="20" t="s">
         <v>76</v>
       </c>
       <c r="E37" s="10" t="s">
@@ -2185,7 +2202,7 @@
       <c r="C38" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="D38" s="19" t="s">
+      <c r="D38" s="20" t="s">
         <v>80</v>
       </c>
       <c r="E38" s="10"/>
@@ -2200,7 +2217,7 @@
       <c r="C39" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="D39" s="19" t="s">
+      <c r="D39" s="20" t="s">
         <v>83</v>
       </c>
       <c r="E39" s="10"/>
@@ -2249,7 +2266,7 @@
       <c r="C42" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="D42" s="19" t="s">
+      <c r="D42" s="20" t="s">
         <v>93</v>
       </c>
       <c r="E42" s="10" t="s">
@@ -2300,7 +2317,7 @@
       <c r="C45" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="D45" s="19" t="s">
+      <c r="D45" s="20" t="s">
         <v>101</v>
       </c>
       <c r="E45" s="10" t="s">
@@ -2317,7 +2334,7 @@
       <c r="C46" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="D46" s="19" t="s">
+      <c r="D46" s="20" t="s">
         <v>104</v>
       </c>
       <c r="E46" s="10"/>
@@ -2349,7 +2366,7 @@
       <c r="C48" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="D48" s="19" t="s">
+      <c r="D48" s="20" t="s">
         <v>110</v>
       </c>
       <c r="E48" s="10" t="s">
@@ -2366,7 +2383,7 @@
       <c r="C49" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="D49" s="19" t="s">
+      <c r="D49" s="20" t="s">
         <v>113</v>
       </c>
       <c r="E49" s="10" t="s">
@@ -2383,7 +2400,7 @@
       <c r="C50" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="D50" s="19" t="s">
+      <c r="D50" s="20" t="s">
         <v>116</v>
       </c>
       <c r="E50" s="10" t="s">
@@ -2477,7 +2494,7 @@
       <c r="C57" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="D57" s="19" t="s">
+      <c r="D57" s="20" t="s">
         <v>130</v>
       </c>
       <c r="E57" s="10"/>
@@ -2493,7 +2510,7 @@
       <c r="C58" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D58" s="19" t="s">
+      <c r="D58" s="20" t="s">
         <v>133</v>
       </c>
       <c r="E58" s="10"/>
@@ -2597,7 +2614,7 @@
       <c r="C64" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="D64" s="19" t="s">
+      <c r="D64" s="20" t="s">
         <v>153</v>
       </c>
       <c r="E64" s="10"/>
@@ -2629,7 +2646,7 @@
       <c r="C66" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="D66" s="19" t="s">
+      <c r="D66" s="20" t="s">
         <v>159</v>
       </c>
       <c r="E66" s="10"/>
@@ -2645,7 +2662,7 @@
       <c r="C67" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="D67" s="19" t="s">
+      <c r="D67" s="20" t="s">
         <v>162</v>
       </c>
       <c r="E67" s="10"/>
@@ -2659,7 +2676,7 @@
         <v>163</v>
       </c>
       <c r="C68" s="15"/>
-      <c r="D68" s="19" t="s">
+      <c r="D68" s="20" t="s">
         <v>164</v>
       </c>
       <c r="E68" s="10"/>
@@ -2674,12 +2691,42 @@
       <c r="C69" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="D69" s="19" t="s">
+      <c r="D69" s="20" t="s">
         <v>166</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>147</v>
       </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="14">
+        <v>15</v>
+      </c>
+      <c r="B70" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C70" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="D70" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="E70" s="18"/>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="14">
+        <v>16</v>
+      </c>
+      <c r="B71" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="C71" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="D71" s="21" t="s">
+        <v>171</v>
+      </c>
+      <c r="E71" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
10 DECEMBER 2025 CLOSING
</commit_message>
<xml_diff>
--- a/SUPPLIER RELATED/Phone Book BALAGAN.xlsx
+++ b/SUPPLIER RELATED/Phone Book BALAGAN.xlsx
@@ -72,7 +72,8 @@
             <rFont val="Times New Roman"/>
             <charset val="0"/>
           </rPr>
-          <t>Cape discovery (wine)</t>
+          <t>Cape discovery (wine)
+Jim Beam</t>
         </r>
       </text>
     </comment>
@@ -152,7 +153,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="173">
   <si>
     <t>BALAGAN RESTO &amp; LOUNGE BAR</t>
   </si>
@@ -521,6 +522,9 @@
   </si>
   <si>
     <t>0813-3847-4143</t>
+  </si>
+  <si>
+    <t>Nano Dewata</t>
   </si>
   <si>
     <t>KITCHEN</t>
@@ -847,12 +851,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
@@ -1337,7 +1341,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1386,12 +1390,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1711,7 +1713,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="5.08571428571429" style="2" customWidth="1"/>
@@ -1824,7 +1826,7 @@
       <c r="C10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="10"/>
@@ -1887,7 +1889,7 @@
       <c r="C16" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="10" t="s">
@@ -1919,7 +1921,7 @@
       <c r="C18" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>31</v>
       </c>
       <c r="E18" s="10"/>
@@ -2134,7 +2136,7 @@
       <c r="C34" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="D34" s="19" t="s">
         <v>66</v>
       </c>
       <c r="E34" s="10" t="s">
@@ -2151,7 +2153,7 @@
       <c r="C35" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="D35" s="19" t="s">
         <v>70</v>
       </c>
       <c r="E35" s="10" t="s">
@@ -2168,7 +2170,7 @@
       <c r="C36" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="20" t="s">
+      <c r="D36" s="19" t="s">
         <v>73</v>
       </c>
       <c r="E36" s="10" t="s">
@@ -2185,7 +2187,7 @@
       <c r="C37" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="D37" s="20" t="s">
+      <c r="D37" s="19" t="s">
         <v>76</v>
       </c>
       <c r="E37" s="10" t="s">
@@ -2202,7 +2204,7 @@
       <c r="C38" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="D38" s="20" t="s">
+      <c r="D38" s="19" t="s">
         <v>80</v>
       </c>
       <c r="E38" s="10"/>
@@ -2217,7 +2219,7 @@
       <c r="C39" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="19" t="s">
         <v>83</v>
       </c>
       <c r="E39" s="10"/>
@@ -2266,7 +2268,7 @@
       <c r="C42" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="D42" s="20" t="s">
+      <c r="D42" s="19" t="s">
         <v>93</v>
       </c>
       <c r="E42" s="10" t="s">
@@ -2317,7 +2319,7 @@
       <c r="C45" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="D45" s="20" t="s">
+      <c r="D45" s="19" t="s">
         <v>101</v>
       </c>
       <c r="E45" s="10" t="s">
@@ -2334,7 +2336,7 @@
       <c r="C46" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="D46" s="20" t="s">
+      <c r="D46" s="19" t="s">
         <v>104</v>
       </c>
       <c r="E46" s="10"/>
@@ -2366,7 +2368,7 @@
       <c r="C48" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="D48" s="20" t="s">
+      <c r="D48" s="19" t="s">
         <v>110</v>
       </c>
       <c r="E48" s="10" t="s">
@@ -2383,7 +2385,7 @@
       <c r="C49" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="D49" s="20" t="s">
+      <c r="D49" s="19" t="s">
         <v>113</v>
       </c>
       <c r="E49" s="10" t="s">
@@ -2400,7 +2402,7 @@
       <c r="C50" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="D50" s="20" t="s">
+      <c r="D50" s="19" t="s">
         <v>116</v>
       </c>
       <c r="E50" s="10" t="s">
@@ -2437,302 +2439,312 @@
       </c>
       <c r="E52" s="10"/>
     </row>
-    <row r="53" spans="2:4">
-      <c r="B53" s="17"/>
+    <row r="53" spans="1:4">
+      <c r="A53" s="2">
+        <v>22</v>
+      </c>
+      <c r="B53" s="17" t="s">
+        <v>123</v>
+      </c>
       <c r="C53" s="17"/>
       <c r="D53" s="17"/>
     </row>
-    <row r="54" spans="1:5">
-      <c r="A54" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
+    <row r="54" spans="2:4">
+      <c r="B54" s="17"/>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B55" s="11"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="11"/>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B55" s="13" t="s">
+      <c r="B56" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13" t="s">
+      <c r="C56" s="13"/>
+      <c r="D56" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E55" s="13" t="s">
+      <c r="E56" s="13" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5">
-      <c r="A56" s="14">
-        <v>1</v>
-      </c>
-      <c r="B56" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="C56" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="D56" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="14">
-        <f t="shared" ref="A57:A68" si="0">A56+1</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B57" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="D57" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="E57" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C57" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="D57" s="20" t="s">
-        <v>130</v>
-      </c>
-      <c r="E57" s="10"/>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="14">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f t="shared" ref="A58:A69" si="0">A57+1</f>
+        <v>2</v>
       </c>
       <c r="B58" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="D58" s="19" t="s">
         <v>131</v>
-      </c>
-      <c r="C58" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="D58" s="20" t="s">
-        <v>133</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="14">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B59" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D59" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="C59" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="D59" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="E59" s="10" t="s">
-        <v>10</v>
-      </c>
+      <c r="E59" s="10"/>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="14">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C60" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D60" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="D60" s="15" t="s">
-        <v>138</v>
-      </c>
       <c r="E60" s="10" t="s">
-        <v>139</v>
+        <v>10</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="14">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B61" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="D61" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="E61" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="C61" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="D61" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="14">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B62" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D62" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="E62" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="C62" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="D62" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="14">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B63" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="C63" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="D63" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="E63" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="C63" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="D63" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E63" s="10"/>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="14">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B64" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="C64" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="D64" s="15" t="s">
         <v>151</v>
-      </c>
-      <c r="C64" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="D64" s="20" t="s">
-        <v>153</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="14">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B65" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="C65" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="D65" s="19" t="s">
         <v>154</v>
-      </c>
-      <c r="C65" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="D65" s="15" t="s">
-        <v>156</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="14">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B66" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="C66" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="D66" s="15" t="s">
         <v>157</v>
-      </c>
-      <c r="C66" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="D66" s="20" t="s">
-        <v>159</v>
       </c>
       <c r="E66" s="10"/>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="14">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B67" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="C67" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="D67" s="19" t="s">
         <v>160</v>
-      </c>
-      <c r="C67" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="D67" s="20" t="s">
-        <v>162</v>
       </c>
       <c r="E67" s="10"/>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="14">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B68" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="C68" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D68" s="19" t="s">
         <v>163</v>
-      </c>
-      <c r="C68" s="15"/>
-      <c r="D68" s="20" t="s">
-        <v>164</v>
       </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="14">
-        <v>14</v>
-      </c>
-      <c r="B69" s="10" t="s">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="B69" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="C69" s="15"/>
+      <c r="D69" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="C69" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="D69" s="20" t="s">
-        <v>166</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>147</v>
-      </c>
+      <c r="E69" s="10"/>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" s="14">
-        <v>15</v>
-      </c>
-      <c r="B70" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B70" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="C70" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D70" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="C70" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="D70" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="E70" s="18"/>
+      <c r="E70" s="10" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="14">
+        <v>15</v>
+      </c>
+      <c r="B71" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="C71" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="D71" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E71" s="10"/>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="14">
         <v>16</v>
       </c>
-      <c r="B71" s="18" t="s">
-        <v>170</v>
-      </c>
-      <c r="C71" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="D71" s="21" t="s">
+      <c r="B72" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="E71" s="18"/>
+      <c r="C72" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="D72" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E72" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A55:E55"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId3" display="balagan.uluwatu@gmail.com"/>

</xml_diff>